<commit_message>
update downloads information for people to know about files
</commit_message>
<xml_diff>
--- a/05_manuscript/dataset_list.xlsx
+++ b/05_manuscript/dataset_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C60"/>
+  <dimension ref="A1:D101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -424,10 +424,15 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Parts</t>
+          <t>Part</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
         <is>
           <t>DOI</t>
         </is>
@@ -444,6 +449,11 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>60 files (dim 50,100,200,300,500; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>10.5281/zenodo.17328169</t>
         </is>
       </c>
@@ -455,33 +465,43 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Part 1: 10.5281/zenodo.17329023; Part 2: 10.5281/zenodo.17334562</t>
+          <t>45 files (dim 50,100,200,300; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17329023</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>bg</t>
+          <t>ar</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>10.5281/zenodo.17430982</t>
+          <t>15 files (dim 300,500; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17334562</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>bn</t>
+          <t>bg</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -489,14 +509,19 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>10.5281/zenodo.17442281</t>
+          <t>60 files (dim 50,100,200,300,500; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17430982</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>br</t>
+          <t>bn</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -504,14 +529,19 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>10.5281/zenodo.17443001</t>
+          <t>60 files (dim 50,100,200,300,500; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17442281</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>bs</t>
+          <t>br</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -519,14 +549,19 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>10.5281/zenodo.17344027</t>
+          <t>60 files (dim 50,100,200,300,500; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17443001</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ca</t>
+          <t>bs</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -534,29 +569,39 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>10.5281/zenodo.17352129</t>
+          <t>60 files (dim 50,100,200,300,500; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17344027</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>cs</t>
+          <t>ca</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Part 1: 10.5281/zenodo.17371745; Part 2: 10.5281/zenodo.17386111</t>
+          <t>60 files (dim 50,100,200,300,500; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17352129</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>da</t>
+          <t>cs</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -564,74 +609,99 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>10.5281/zenodo.17389059</t>
+          <t>50 files (dim 50,100,200,300,500; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17371745</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>cs</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Part 1: 10.5281/zenodo.17443203; Part 2: 10.5281/zenodo.17446694; Part 3: 10.5281/zenodo.17449490; Part 4: 10.5281/zenodo.17482872</t>
+          <t>10 files (dim 500; window 2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17386111</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>el</t>
+          <t>da</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Part 1: 10.5281/zenodo.17390625; Part 2: 10.5281/zenodo.17394622</t>
+          <t>60 files (dim 50,100,200,300,500; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17389059</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>de</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Part 1: 10.5281/zenodo.17361499; Part 2: 10.5281/zenodo.17576288; Part 3: 10.5281/zenodo.17585011; Part 4: 10.5281/zenodo.17595213; Part 5: 10.5281/zenodo.17603186; Part 6: 10.5281/zenodo.17618269; Part 7: 10.5281/zenodo.17619406; Part 8: 10.5281/zenodo.17619964; Part 9: 10.5281/zenodo.17620219; Part 10: 10.5281/zenodo.17620246</t>
+          <t>33 files (dim 50,100,200; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17443203</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>eo</t>
+          <t>de</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>10.5281/zenodo.17394831</t>
+          <t>13 files (dim 200,300; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17446694</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>es</t>
+          <t>de</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -639,29 +709,39 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Part 1: 10.5281/zenodo.17450685; Part 2: 10.5281/zenodo.17459793; Part 3: 10.5281/zenodo.17468301</t>
+          <t>7 files (dim 300,500; window 1,2,3,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17449490</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>et</t>
+          <t>de</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>10.5281/zenodo.17403307</t>
+          <t>7 files (dim 500; window 3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17482872</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>eu</t>
+          <t>el</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -669,194 +749,259 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>10.5281/zenodo.17422512</t>
+          <t>58 files (dim 50,100,200,300,500; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17390625</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>fa</t>
+          <t>el</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>10.5281/zenodo.17503241</t>
+          <t>2 files (dim 500; window 6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17394622</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>fi</t>
+          <t>en</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Part 1: 10.5281/zenodo.17496255; Part 2: 10.5281/zenodo.17501942</t>
+          <t>20 files (dim 50,100; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17361499</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>en</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>10.5281/zenodo.17337550</t>
+          <t>9 files (dim 100,200; window 1,2,3,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17576288</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>gl</t>
+          <t>en</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>10.5281/zenodo.17343732</t>
+          <t>7 files (dim 200; window 3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17585011</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>he</t>
+          <t>en</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Part 1: 10.5281/zenodo.17366566; Part 2: 10.5281/zenodo.17435642</t>
+          <t>5 files (dim 300; window 1,2,3; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17595213</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>hi</t>
+          <t>en</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>10.5281/zenodo.17506770</t>
+          <t>5 files (dim 300; window 3,4,5; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17603186</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>hr</t>
+          <t>en</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Part 1: 10.5281/zenodo.17507139; Part 2: 10.5281/zenodo.17510398</t>
+          <t>3 files (dim 300,500; window 1,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17618269</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>hu</t>
+          <t>en</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Part 1: 10.5281/zenodo.17450130; Part 2: 10.5281/zenodo.17487438; Part 3: 10.5281/zenodo.17495349</t>
+          <t>3 files (dim 500; window 1,2; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17619406</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>hy</t>
+          <t>en</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>10.5281/zenodo.17503079</t>
+          <t>3 files (dim 500; window 3,4; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17619964</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>en</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>10.5281/zenodo.17508548</t>
+          <t>3 files (dim 500; window 4,5; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17620219</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>is</t>
+          <t>en</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>10.5281/zenodo.17512316</t>
+          <t>2 files (dim 500; window 6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17620246</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>it</t>
+          <t>eo</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Part 1: 10.5281/zenodo.17517234; Part 2: 10.5281/zenodo.17520185; Part 3: 10.5281/zenodo.17531837</t>
+          <t>60 files (dim 50,100,200,300,500; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17394831</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>es</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -864,59 +1009,79 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>10.5281/zenodo.17539310</t>
+          <t>41 files (dim 50,100,200,300; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17450685</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ka</t>
+          <t>es</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>10.5281/zenodo.17548848</t>
+          <t>14 files (dim 300,500; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17459793</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>kk</t>
+          <t>es</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>10.5281/zenodo.17551941</t>
+          <t>5 files (dim 500; window 4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17468301</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ko</t>
+          <t>et</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Part 1: 10.5281/zenodo.17553195; Part 2: 10.5281/zenodo.17558872</t>
+          <t>60 files (dim 50,100,200,300,500; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17403307</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>lt</t>
+          <t>eu</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -924,14 +1089,19 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>10.5281/zenodo.17559525</t>
+          <t>60 files (dim 50,100,200,300,500; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17422512</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>lv</t>
+          <t>fa</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -939,14 +1109,19 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>10.5281/zenodo.17560572</t>
+          <t>60 files (dim 50,100,200,300,500; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17503241</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>mk</t>
+          <t>fi</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -954,29 +1129,39 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>10.5281/zenodo.17561123</t>
+          <t>50 files (dim 50,100,200,300,500; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17496255</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>ml</t>
+          <t>fi</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>10.5281/zenodo.17562308</t>
+          <t>10 files (dim 500; window 2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17501942</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>ms</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -984,29 +1169,39 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>10.5281/zenodo.17562936</t>
+          <t>60 files (dim 50,100,200,300,500; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17337550</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>gl</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Part 1: 10.5281/zenodo.17563962; Part 2: 10.5281/zenodo.17566504</t>
+          <t>60 files (dim 50,100,200,300,500; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17343732</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>he</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1014,74 +1209,99 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>10.5281/zenodo.17566092</t>
+          <t>58 files (dim 50,100,200,300,500; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17366566</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>pl</t>
+          <t>he</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Part 1: 10.5281/zenodo.17575147; Part 2: 10.5281/zenodo.17577928; Part 3: 10.5281/zenodo.17586413</t>
+          <t>2 files (dim 500; window 6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17435642</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>pt</t>
+          <t>hi</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Part 1: 10.5281/zenodo.17582531; Part 2: 10.5281/zenodo.17605883</t>
+          <t>60 files (dim 50,100,200,300,500; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17506770</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>ro</t>
+          <t>hr</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Part 1: 10.5281/zenodo.17586582; Part 2: 10.5281/zenodo.17596253</t>
+          <t>56 files (dim 50,100,200,300,500; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17507139</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>ru</t>
+          <t>hr</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Part 1: 10.5281/zenodo.17593827; Part 2: 10.5281/zenodo.17603392; Part 3: 10.5281/zenodo.17606023</t>
+          <t>4 files (dim 500; window 5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17510398</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>si</t>
+          <t>hu</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1089,44 +1309,59 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>10.5281/zenodo.17559974</t>
+          <t>44 files (dim 50,100,200,300; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17450130</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>sk</t>
+          <t>hu</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>10.5281/zenodo.17555316</t>
+          <t>14 files (dim 300,500; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17487438</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>sl</t>
+          <t>hu</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>10.5281/zenodo.17560097</t>
+          <t>2 files (dim 500; window 6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17495349</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>sq</t>
+          <t>hy</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1134,44 +1369,59 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>10.5281/zenodo.17602011</t>
+          <t>60 files (dim 50,100,200,300,500; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17503079</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>sr</t>
+          <t>id</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Part 1: 10.5281/zenodo.17615164; Part 2: 10.5281/zenodo.17615219; Part 3: 10.5281/zenodo.17615221</t>
+          <t>60 files (dim 50,100,200,300,500; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17508548</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>sv</t>
+          <t>is</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Part 1: 10.5281/zenodo.17561217; Part 2: 10.5281/zenodo.17561268; Part 3: 10.5281/zenodo.17561285</t>
+          <t>60 files (dim 50,100,200,300,500; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17512316</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>ta</t>
+          <t>it</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1179,44 +1429,59 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>10.5281/zenodo.17616704</t>
+          <t>46 files (dim 50,100,200,300; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17517234</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>te</t>
+          <t>it</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>10.5281/zenodo.17618540</t>
+          <t>7 files (dim 300,500; window 1,2,3,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17520185</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>th</t>
+          <t>it</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>10.5281/zenodo.17621048</t>
+          <t>7 files (dim 500; window 3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17531837</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>tl</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1224,29 +1489,39 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>10.5281/zenodo.17623253</t>
+          <t>60 files (dim 50,100,200,300,500; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17539310</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>tr</t>
+          <t>ka</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Part 1: 10.5281/zenodo.17622011; Part 2: 10.5281/zenodo.17625108</t>
+          <t>60 files (dim 50,100,200,300,500; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17548848</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>tw</t>
+          <t>kk</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1254,67 +1529,912 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>10.5281/zenodo.17466332</t>
+          <t>60 files (dim 50,100,200,300,500; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17551941</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>uk</t>
+          <t>ko</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Part 1: 10.5281/zenodo.17624050; Part 2: 10.5281/zenodo.17635267</t>
+          <t>55 files (dim 50,100,200,300,500; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17553195</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>ur</t>
+          <t>ko</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>10.5281/zenodo.17624311</t>
+          <t>5 files (dim 500; window 4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17558872</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>vi</t>
+          <t>lt</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Part 1: 10.5281/zenodo.17639257; Part 2: 10.5281/zenodo.17642074; Part 3: 10.5281/zenodo.17648757; Part 4: 10.5281/zenodo.17657125</t>
+          <t>60 files (dim 50,100,200,300,500; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17559525</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
+          <t>lv</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>1</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>60 files (dim 50,100,200,300,500; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17560572</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>mk</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>1</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>60 files (dim 50,100,200,300,500; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17561123</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>1</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>60 files (dim 50,100,200,300,500; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17562308</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>ms</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>1</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>60 files (dim 50,100,200,300,500; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17562936</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>1</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>48 files (dim 50,100,200,300; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17563962</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>2</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>12 files (dim 500; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17566504</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>1</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>60 files (dim 50,100,200,300,500; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17566092</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>pl</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>1</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>42 files (dim 50,100,200,300; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17575147</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>pl</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>2</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>15 files (dim 300,500; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17577928</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>pl</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>3</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>3 files (dim 500; window 5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17586413</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>pt</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>1</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>53 files (dim 50,100,200,300,500; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17582531</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>pt</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>2</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>7 files (dim 500; window 3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17605883</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>ro</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>1</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>58 files (dim 50,100,200,300,500; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17586582</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>ro</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>2</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>2 files (dim 500; window 6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17596253</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>ru</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>1</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>38 files (dim 50,100,200,300; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17593827</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>ru</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>2</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>13 files (dim 300,500; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17603392</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>ru</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>3</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>9 files (dim 500; window 2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17606023</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>1</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>60 files (dim 50,100,200,300,500; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17559974</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>sk</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>1</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>60 files (dim 50,100,200,300,500; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17555316</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>sl</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>1</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>60 files (dim 50,100,200,300,500; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17560097</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>sq</t>
+        </is>
+      </c>
+      <c r="B80" t="n">
+        <v>1</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>60 files (dim 50,100,200,300,500; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17602011</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>sr</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>1</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>41 files (dim 50,100,200,300; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17615164</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>sr</t>
+        </is>
+      </c>
+      <c r="B82" t="n">
+        <v>2</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>14 files (dim 300,500; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17615219</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>sr</t>
+        </is>
+      </c>
+      <c r="B83" t="n">
+        <v>3</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>5 files (dim 500; window 4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17615221</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>sv</t>
+        </is>
+      </c>
+      <c r="B84" t="n">
+        <v>1</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>36 files (dim 50,100,200; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17561217</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>sv</t>
+        </is>
+      </c>
+      <c r="B85" t="n">
+        <v>2</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>12 files (dim 300; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17561268</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>sv</t>
+        </is>
+      </c>
+      <c r="B86" t="n">
+        <v>3</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>12 files (dim 500; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17561285</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>te</t>
+        </is>
+      </c>
+      <c r="B87" t="n">
+        <v>1</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>60 files (dim 50,100,200,300,500; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17618540</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>th</t>
+        </is>
+      </c>
+      <c r="B88" t="n">
+        <v>1</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>60 files (dim 50,100,200,300,500; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17621048</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>tl</t>
+        </is>
+      </c>
+      <c r="B89" t="n">
+        <v>1</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>60 files (dim 50,100,200,300,500; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17623253</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>tr</t>
+        </is>
+      </c>
+      <c r="B90" t="n">
+        <v>1</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>49 files (dim 50,100,200,300,500; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17622011</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>tr</t>
+        </is>
+      </c>
+      <c r="B91" t="n">
+        <v>2</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>11 files (dim 500; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17625108</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>tw</t>
+        </is>
+      </c>
+      <c r="B92" t="n">
+        <v>1</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>60 files (dim 50,100,200,300,500; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17466332</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>uk</t>
+        </is>
+      </c>
+      <c r="B93" t="n">
+        <v>1</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>51 files (dim 50,100,200,300,500; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17624050</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>uk</t>
+        </is>
+      </c>
+      <c r="B94" t="n">
+        <v>2</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>9 files (dim 500; window 2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17635267</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>ur</t>
+        </is>
+      </c>
+      <c r="B95" t="n">
+        <v>1</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>60 files (dim 50,100,200,300,500; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17624311</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>vi</t>
+        </is>
+      </c>
+      <c r="B96" t="n">
+        <v>1</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>32 files (dim 50,100,200; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17639257</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>vi</t>
+        </is>
+      </c>
+      <c r="B97" t="n">
+        <v>2</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>13 files (dim 200,300; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17642074</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>vi</t>
+        </is>
+      </c>
+      <c r="B98" t="n">
+        <v>3</v>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>8 files (dim 300,500; window 1,2,3,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17648757</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>vi</t>
+        </is>
+      </c>
+      <c r="B99" t="n">
+        <v>4</v>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>7 files (dim 500; window 3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17657125</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
           <t>zh</t>
         </is>
       </c>
-      <c r="B60" t="n">
+      <c r="B100" t="n">
+        <v>1</v>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>48 files (dim 50,100,200,300; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17478882</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>zh</t>
+        </is>
+      </c>
+      <c r="B101" t="n">
         <v>2</v>
       </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>Part 1: 10.5281/zenodo.17478882; Part 2: 10.5281/zenodo.17610765</t>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>12 files (dim 500; window 1,2,3,4,5,6; cbow,sg)</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.17610765</t>
         </is>
       </c>
     </row>

</xml_diff>